<commit_message>
Added paper images and updated Fishpond Monitoring System v2
</commit_message>
<xml_diff>
--- a/IoT-Based Fishpond Monitoring System/version 2/BOM.xlsx
+++ b/IoT-Based Fishpond Monitoring System/version 2/BOM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DELL\Desktop\cnic\Projects info\fish pond\version 2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\Projects info\IoT-Based Fishpond Monitoring System\version 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C57665F5-91C1-456A-8F5F-116C20866899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E6E405-B11E-4D64-A814-02416506C06F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{15628D95-0D6F-4CFE-9129-88278DE76781}"/>
   </bookViews>
@@ -50,9 +50,6 @@
     <t>website</t>
   </si>
   <si>
-    <t>Esp32</t>
-  </si>
-  <si>
     <t>ph-sensor</t>
   </si>
   <si>
@@ -93,6 +90,9 @@
   </si>
   <si>
     <t>Ultrasonic Sensor</t>
+  </si>
+  <si>
+    <t>Camera</t>
   </si>
 </sst>
 </file>
@@ -510,27 +510,27 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>4</v>
+        <v>18</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="D2">
-        <v>1150</v>
+        <v>10050</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="D3">
         <v>5000</v>
@@ -538,13 +538,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D4">
         <v>280</v>
@@ -552,13 +552,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D5">
         <v>2300</v>
@@ -566,13 +566,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B6">
+        <v>1</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>13</v>
-      </c>
-      <c r="B6">
-        <v>1</v>
-      </c>
-      <c r="C6" s="1" t="s">
-        <v>14</v>
       </c>
       <c r="D6">
         <v>35000</v>
@@ -580,13 +580,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7">
+        <v>1</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>15</v>
-      </c>
-      <c r="B7">
-        <v>1</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="D7">
         <v>1100</v>
@@ -594,13 +594,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="D8">
         <v>1250</v>
@@ -608,11 +608,11 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C12" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="D12" s="3">
         <f>SUM(D2:D8)</f>
-        <v>46080</v>
+        <v>54980</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added images for fish v2 and rename repo
</commit_message>
<xml_diff>
--- a/IoT-Based Fishpond Monitoring System/version 2/BOM.xlsx
+++ b/IoT-Based Fishpond Monitoring System/version 2/BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Personal\Projects info\IoT-Based Fishpond Monitoring System\version 2\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87E6E405-B11E-4D64-A814-02416506C06F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{77D5ED40-DEF6-443C-A368-DA2DB524F122}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11160" xr2:uid="{15628D95-0D6F-4CFE-9129-88278DE76781}"/>
+    <workbookView xWindow="1170" yWindow="1170" windowWidth="15375" windowHeight="7875" xr2:uid="{15628D95-0D6F-4CFE-9129-88278DE76781}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="19">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
   <si>
     <t>Name</t>
   </si>
@@ -44,9 +44,6 @@
     <t>Quantity</t>
   </si>
   <si>
-    <t>price</t>
-  </si>
-  <si>
     <t>website</t>
   </si>
   <si>
@@ -59,9 +56,6 @@
     <t xml:space="preserve"> Tsw-20m</t>
   </si>
   <si>
-    <t>https://electrobes.com/product/esp32-wroom-32-38-pins-wifibluetooth-mcu-module/</t>
-  </si>
-  <si>
     <t>Liquid pH Sensor pH Electrode Probe For Arduino in Pakistan</t>
   </si>
   <si>
@@ -92,17 +86,30 @@
     <t>Ultrasonic Sensor</t>
   </si>
   <si>
-    <t>Camera</t>
+    <t>Color Sensosr</t>
+  </si>
+  <si>
+    <t>TCS34725 Color Sensor Module in Pakistan | Electronics Hub</t>
+  </si>
+  <si>
+    <t>Hardware Cost</t>
+  </si>
+  <si>
+    <t>USD   173.75</t>
+  </si>
+  <si>
+    <t>Price in PKR</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="1">
+  <numFmts count="2">
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="164" formatCode="_([$PKR]\ * #,##0.00_);_([$PKR]\ * \(#,##0.00\);_([$PKR]\ * &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -126,6 +133,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="7" tint="-0.249977111117893"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -144,17 +166,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1" applyFont="1"/>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
@@ -488,9 +514,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D0290EB5-439A-4485-A355-A5E3C8932CC9}">
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="17" customWidth="1"/>
     <col min="4" max="4" width="14.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -502,35 +529,30 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>18</v>
       </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>7</v>
-      </c>
+      <c r="C2" s="1"/>
       <c r="D2">
-        <v>10050</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B3">
         <v>1</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D3">
         <v>5000</v>
@@ -538,13 +560,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B4">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="D4">
         <v>280</v>
@@ -552,13 +574,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B5">
         <v>1</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="D5">
         <v>2300</v>
@@ -566,13 +588,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B6">
         <v>1</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6">
         <v>35000</v>
@@ -580,13 +602,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B7">
         <v>1</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7">
         <v>1100</v>
@@ -594,36 +616,55 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B8">
         <v>1</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="D8">
         <v>1250</v>
       </c>
     </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>16</v>
+      </c>
+      <c r="B9">
+        <v>1</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="D9">
+        <v>950</v>
+      </c>
+    </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="C12" s="2" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="D12" s="3">
-        <f>SUM(D2:D8)</f>
-        <v>54980</v>
+        <f>SUM(D2:D9)</f>
+        <v>47780</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="D13" s="5" t="s">
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{EF1CF07E-149A-4FBC-BEF6-E2CD13C53D7A}"/>
-    <hyperlink ref="C3" r:id="rId2" display="https://electrobes.com/product/liquid-ph-sensor-with-bnc-ph-electrode-probe-for-arduino/" xr:uid="{1B41358D-466D-4B87-BAEE-3DD5631FAD12}"/>
-    <hyperlink ref="C5" r:id="rId3" display="https://electrobes.com/product/water-turbidity-sensor-with-analog-output-module/" xr:uid="{33875481-4278-454D-8484-FDDD97DD026B}"/>
-    <hyperlink ref="C4" r:id="rId4" display="https://electrobes.com/product/ds18b20-waterproof-temperature-sensor/" xr:uid="{13F82AA0-F41B-44A5-93B8-1FE45DDCE1A1}"/>
-    <hyperlink ref="C6" r:id="rId5" display="https://electrobes.com/?s=raspberry+pi+5&amp;post_type=product" xr:uid="{7F15278F-F63E-4213-B62C-938220116BAA}"/>
-    <hyperlink ref="C7" r:id="rId6" display="https://electrobes.com/product/tds-meter-v1-0-module-water-quality-sensor-for-arduino/" xr:uid="{04F3463F-E2CE-4A9A-BC41-6D4872BAFC88}"/>
-    <hyperlink ref="C8" r:id="rId7" display="https://electrobes.com/product/jsn-sr04t-waterproof-ultrasonic-sensor-module/" xr:uid="{E09179DB-EAEE-4DED-BF7B-C254B6A9E690}"/>
+    <hyperlink ref="C3" r:id="rId1" display="https://electrobes.com/product/liquid-ph-sensor-with-bnc-ph-electrode-probe-for-arduino/" xr:uid="{1B41358D-466D-4B87-BAEE-3DD5631FAD12}"/>
+    <hyperlink ref="C5" r:id="rId2" display="https://electrobes.com/product/water-turbidity-sensor-with-analog-output-module/" xr:uid="{33875481-4278-454D-8484-FDDD97DD026B}"/>
+    <hyperlink ref="C4" r:id="rId3" display="https://electrobes.com/product/ds18b20-waterproof-temperature-sensor/" xr:uid="{13F82AA0-F41B-44A5-93B8-1FE45DDCE1A1}"/>
+    <hyperlink ref="C6" r:id="rId4" display="https://electrobes.com/?s=raspberry+pi+5&amp;post_type=product" xr:uid="{7F15278F-F63E-4213-B62C-938220116BAA}"/>
+    <hyperlink ref="C7" r:id="rId5" display="https://electrobes.com/product/tds-meter-v1-0-module-water-quality-sensor-for-arduino/" xr:uid="{04F3463F-E2CE-4A9A-BC41-6D4872BAFC88}"/>
+    <hyperlink ref="C8" r:id="rId6" display="https://electrobes.com/product/jsn-sr04t-waterproof-ultrasonic-sensor-module/" xr:uid="{E09179DB-EAEE-4DED-BF7B-C254B6A9E690}"/>
+    <hyperlink ref="C9" r:id="rId7" display="https://electronicshub.pk/product/tcs34725-color-sensor-module/" xr:uid="{B36ECD88-32EB-4673-A2A0-1AC3290029BC}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId8"/>

</xml_diff>